<commit_message>
Refactoring and Terminal UI
</commit_message>
<xml_diff>
--- a/Entries HBC Premier Elite 2024.xlsx
+++ b/Entries HBC Premier Elite 2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sofienystrom/Badminton-Timetable-Solver/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E02814-FDC4-CD48-AF21-2F15B1E459EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BEDACC-CE42-614E-A77C-25A87035A215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="29400" windowHeight="16680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Entries HBC Premier Elite 2024" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Rule Violations" sheetId="4" r:id="rId4"/>
     <sheet name="Event Analysis" sheetId="5" r:id="rId5"/>
     <sheet name="timetable-12 40" sheetId="6" r:id="rId6"/>
-    <sheet name="timetable" sheetId="7" r:id="rId7"/>
+    <sheet name="timetable_old_version" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>

<commit_message>
New logic for entering time of tournament, and umpire_chair variable
</commit_message>
<xml_diff>
--- a/Entries HBC Premier Elite 2024.xlsx
+++ b/Entries HBC Premier Elite 2024.xlsx
@@ -26244,7 +26244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="27.83203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -26898,6 +26898,27 @@
       <c r="A65" t="inlineStr">
         <is>
           <t>Log entry at 2026-10-19 13:41:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Log entry at 2026-10-19 20:37:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Log entry at 2026-10-19 20:38:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Log entry at 2026-10-19 20:38:49</t>
         </is>
       </c>
     </row>
@@ -32365,7 +32386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B3:AY52"/>
+  <dimension ref="B3:AY70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -32619,194 +32640,179 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="58" t="inlineStr">
+      <c r="D4" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="F4" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F4" s="61" t="inlineStr">
+      <c r="H4" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="J4" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L4" s="61" t="inlineStr">
         <is>
           <t>WD A - 1</t>
         </is>
       </c>
-      <c r="H4" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="J4" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="K4" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="L4" s="69" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="M4" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="N4" s="61" t="inlineStr">
+      <c r="N4" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="O4" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="P4" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="R4" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="T4" s="56" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="V4" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="W4" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="X4" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="Y4" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z4" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AA4" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AB4" s="56" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AC4" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="AD4" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AE4" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AF4" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+      <c r="AG4" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AH4" s="61" t="inlineStr">
         <is>
           <t>WD A - 2</t>
         </is>
       </c>
-      <c r="P4" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R4" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T4" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="U4" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="V4" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="X4" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="Y4" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="Z4" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AA4" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AB4" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AC4" s="69" t="inlineStr">
-        <is>
-          <t>WS C - 4</t>
-        </is>
-      </c>
-      <c r="AD4" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AE4" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AF4" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="AH4" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ4" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AK4" s="66" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-      <c r="AL4" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="AM4" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
+      <c r="AI4" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 4</t>
+        </is>
+      </c>
+      <c r="AJ4" s="56" t="inlineStr">
+        <is>
+          <t>WD V - 3</t>
+        </is>
+      </c>
+      <c r="AK4" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AL4" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 4</t>
+        </is>
+      </c>
+      <c r="AM4" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
         </is>
       </c>
       <c r="AN4" s="54" t="inlineStr">
         <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-      <c r="AO4" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="AP4" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="AQ4" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AR4" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
+          <t>WS V - 5</t>
+        </is>
+      </c>
+      <c r="AP4" s="66" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AQ4" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 5</t>
+        </is>
+      </c>
+      <c r="AR4" s="56" t="inlineStr">
+        <is>
+          <t>WD V - 4</t>
         </is>
       </c>
       <c r="AS4" s="58" t="inlineStr">
         <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AT4" s="71" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="AU4" s="61" t="inlineStr">
-        <is>
-          <t>WD A - 4</t>
-        </is>
-      </c>
-      <c r="AW4" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 5</t>
-        </is>
-      </c>
-      <c r="AX4" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="AY4" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="AV4" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="AY4" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 4</t>
         </is>
       </c>
     </row>
@@ -32814,184 +32820,169 @@
       <c r="B5" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="58" t="inlineStr">
+      <c r="D5" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="F5" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F5" s="61" t="inlineStr">
+      <c r="H5" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="J5" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L5" s="61" t="inlineStr">
         <is>
           <t>WD A - 1</t>
         </is>
       </c>
-      <c r="H5" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="J5" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="K5" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="L5" s="69" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="M5" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="N5" s="61" t="inlineStr">
+      <c r="N5" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="P5" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="R5" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="T5" s="56" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="V5" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="X5" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="Y5" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z5" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AA5" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AB5" s="56" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AC5" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="AD5" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AE5" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AF5" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+      <c r="AG5" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AH5" s="61" t="inlineStr">
         <is>
           <t>WD A - 2</t>
         </is>
       </c>
-      <c r="P5" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R5" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T5" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="V5" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="X5" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="Y5" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="Z5" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AA5" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AB5" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AC5" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="AD5" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AE5" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AF5" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="AH5" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ5" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AL5" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="AM5" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AN5" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-      <c r="AO5" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="AP5" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="AQ5" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AR5" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
+      <c r="AI5" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 4</t>
+        </is>
+      </c>
+      <c r="AJ5" s="56" t="inlineStr">
+        <is>
+          <t>WD V - 3</t>
+        </is>
+      </c>
+      <c r="AK5" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AL5" s="69" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="AM5" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AN5" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AP5" s="66" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AQ5" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+      <c r="AR5" s="61" t="inlineStr">
+        <is>
+          <t>WD A - 3</t>
         </is>
       </c>
       <c r="AS5" s="58" t="inlineStr">
         <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AT5" s="71" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="AU5" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
-        </is>
-      </c>
-      <c r="AW5" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 4</t>
-        </is>
-      </c>
-      <c r="AX5" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="AY5" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="AV5" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="AY5" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 4</t>
         </is>
       </c>
     </row>
@@ -32999,169 +32990,169 @@
       <c r="B6" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="58" t="inlineStr">
+      <c r="D6" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="F6" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F6" s="61" t="inlineStr">
+      <c r="H6" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="J6" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L6" s="61" t="inlineStr">
         <is>
           <t>WD A - 1</t>
         </is>
       </c>
-      <c r="H6" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="J6" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="L6" s="69" t="inlineStr">
+      <c r="N6" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="P6" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="R6" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="T6" s="56" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="V6" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="X6" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="Y6" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z6" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AA6" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AB6" s="56" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AC6" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="AD6" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AE6" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AF6" s="69" t="inlineStr">
         <is>
           <t>WS C - 2</t>
         </is>
       </c>
-      <c r="M6" s="65" t="inlineStr">
+      <c r="AG6" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AH6" s="61" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AI6" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AJ6" s="66" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="AK6" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AL6" s="69" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="AM6" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AN6" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AP6" s="66" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AQ6" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+      <c r="AR6" s="61" t="inlineStr">
+        <is>
+          <t>WD A - 3</t>
+        </is>
+      </c>
+      <c r="AS6" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
+        </is>
+      </c>
+      <c r="AV6" s="65" t="inlineStr">
         <is>
           <t>MD B - 1</t>
         </is>
       </c>
-      <c r="N6" s="61" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="P6" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R6" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T6" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="V6" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="X6" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="Y6" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="Z6" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AA6" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AB6" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AC6" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="AD6" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AE6" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AF6" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="AH6" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ6" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AL6" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="AM6" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AN6" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AQ6" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AR6" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AS6" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AT6" s="71" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="AU6" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
-        </is>
-      </c>
-      <c r="AW6" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 4</t>
-        </is>
-      </c>
-      <c r="AX6" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="AY6" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
+      <c r="AY6" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 6</t>
         </is>
       </c>
     </row>
@@ -33169,154 +33160,149 @@
       <c r="B7" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="58" t="inlineStr">
+      <c r="D7" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="F7" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F7" s="61" t="inlineStr">
+      <c r="H7" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="J7" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L7" s="61" t="inlineStr">
         <is>
           <t>WD A - 1</t>
         </is>
       </c>
-      <c r="H7" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="J7" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="L7" s="69" t="inlineStr">
+      <c r="N7" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="P7" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="R7" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="T7" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="V7" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="X7" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="Y7" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z7" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AA7" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AB7" s="56" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AC7" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="AD7" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AE7" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AF7" s="69" t="inlineStr">
         <is>
           <t>WS C - 2</t>
         </is>
       </c>
-      <c r="M7" s="65" t="inlineStr">
+      <c r="AG7" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AH7" s="61" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AI7" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AK7" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AM7" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AN7" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AP7" s="66" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AR7" s="69" t="inlineStr">
+        <is>
+          <t>WS C - 4</t>
+        </is>
+      </c>
+      <c r="AS7" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
+        </is>
+      </c>
+      <c r="AV7" s="65" t="inlineStr">
         <is>
           <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="N7" s="61" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="P7" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R7" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T7" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="V7" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="Y7" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="Z7" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AA7" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AB7" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AC7" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="AD7" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AE7" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AF7" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="AH7" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ7" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AL7" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="AM7" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AN7" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AQ7" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AR7" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AS7" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AW7" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 4</t>
-        </is>
-      </c>
-      <c r="AX7" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="AY7" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
         </is>
       </c>
     </row>
@@ -33324,124 +33310,124 @@
       <c r="B8" t="n">
         <v>5</v>
       </c>
-      <c r="D8" s="58" t="inlineStr">
+      <c r="D8" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="F8" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F8" s="61" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="H8" s="68" t="inlineStr">
+      <c r="H8" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="J8" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L8" s="68" t="inlineStr">
         <is>
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="J8" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="M8" s="65" t="inlineStr">
+      <c r="N8" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="P8" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="R8" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="T8" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="V8" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="X8" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="Y8" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z8" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 3</t>
+        </is>
+      </c>
+      <c r="AA8" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AB8" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 4</t>
+        </is>
+      </c>
+      <c r="AC8" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="AD8" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AE8" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AF8" s="69" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AG8" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AI8" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AM8" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AN8" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AV8" s="65" t="inlineStr">
         <is>
           <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="P8" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R8" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T8" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="V8" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="Y8" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="Z8" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AA8" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AB8" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AC8" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="AE8" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AH8" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ8" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AL8" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="AM8" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AN8" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AQ8" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AS8" s="66" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="AW8" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AY8" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
         </is>
       </c>
     </row>
@@ -33449,124 +33435,109 @@
       <c r="B9" t="n">
         <v>6</v>
       </c>
-      <c r="D9" s="58" t="inlineStr">
+      <c r="D9" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="F9" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F9" s="61" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="H9" s="68" t="inlineStr">
+      <c r="H9" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="J9" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L9" s="68" t="inlineStr">
         <is>
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="J9" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="M9" s="65" t="inlineStr">
+      <c r="N9" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="P9" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="R9" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="T9" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="V9" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="X9" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="Y9" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z9" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 3</t>
+        </is>
+      </c>
+      <c r="AA9" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AD9" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AE9" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AF9" s="69" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AG9" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AI9" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AM9" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AV9" s="65" t="inlineStr">
         <is>
           <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="P9" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R9" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T9" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="V9" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="Y9" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="Z9" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AA9" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AB9" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AC9" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="AE9" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AH9" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ9" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AL9" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="AM9" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AN9" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AQ9" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AS9" s="66" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="AW9" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AY9" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
         </is>
       </c>
     </row>
@@ -33574,109 +33545,94 @@
       <c r="B10" t="n">
         <v>7</v>
       </c>
-      <c r="D10" s="58" t="inlineStr">
+      <c r="D10" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="F10" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F10" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="H10" s="68" t="inlineStr">
+      <c r="H10" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="J10" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L10" s="68" t="inlineStr">
         <is>
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="J10" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="M10" s="65" t="inlineStr">
+      <c r="N10" s="54" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="P10" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="R10" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="T10" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="V10" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="X10" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="Y10" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z10" s="69" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="AA10" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AE10" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AG10" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AM10" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AV10" s="65" t="inlineStr">
         <is>
           <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="P10" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R10" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T10" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="V10" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="Y10" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="Z10" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AB10" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AE10" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AH10" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ10" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AL10" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="AM10" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AQ10" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AS10" s="66" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="AW10" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AY10" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
         </is>
       </c>
     </row>
@@ -33684,104 +33640,89 @@
       <c r="B11" t="n">
         <v>8</v>
       </c>
-      <c r="D11" s="58" t="inlineStr">
+      <c r="D11" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="F11" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F11" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="H11" s="68" t="inlineStr">
+      <c r="H11" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="J11" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L11" s="68" t="inlineStr">
         <is>
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="J11" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="M11" s="65" t="inlineStr">
+      <c r="N11" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="P11" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="R11" s="53" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="T11" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="V11" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="Y11" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z11" s="69" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="AA11" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="AE11" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AG11" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="AM11" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AV11" s="65" t="inlineStr">
         <is>
           <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="P11" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R11" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T11" s="54" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="V11" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="Y11" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="Z11" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="AB11" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AE11" s="55" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AH11" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="AJ11" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AL11" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="AM11" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AS11" s="66" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="AW11" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AY11" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
         </is>
       </c>
     </row>
@@ -33789,84 +33730,64 @@
       <c r="B12" t="n">
         <v>9</v>
       </c>
-      <c r="D12" s="58" t="inlineStr">
+      <c r="D12" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="F12" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F12" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="H12" s="68" t="inlineStr">
+      <c r="H12" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="J12" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L12" s="68" t="inlineStr">
         <is>
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="J12" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="M12" s="65" t="inlineStr">
+      <c r="N12" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="P12" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="R12" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="T12" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="V12" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="AE12" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AV12" s="65" t="inlineStr">
         <is>
           <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="P12" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R12" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T12" s="69" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="V12" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="AB12" s="61" t="inlineStr">
-        <is>
-          <t>WD A - 3</t>
-        </is>
-      </c>
-      <c r="AE12" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AH12" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="AJ12" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AS12" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AW12" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AY12" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
         </is>
       </c>
     </row>
@@ -33874,84 +33795,64 @@
       <c r="B13" t="n">
         <v>10</v>
       </c>
-      <c r="D13" s="58" t="inlineStr">
+      <c r="D13" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="F13" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F13" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="H13" s="68" t="inlineStr">
+      <c r="H13" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="J13" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L13" s="68" t="inlineStr">
         <is>
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="J13" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="M13" s="65" t="inlineStr">
+      <c r="N13" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="P13" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="R13" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="T13" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="V13" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="AE13" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="AV13" s="65" t="inlineStr">
         <is>
           <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="P13" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R13" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T13" s="69" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="V13" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="AB13" s="61" t="inlineStr">
-        <is>
-          <t>WD A - 3</t>
-        </is>
-      </c>
-      <c r="AE13" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AH13" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="AJ13" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AS13" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AW13" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AY13" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
         </is>
       </c>
     </row>
@@ -33959,74 +33860,59 @@
       <c r="B14" t="n">
         <v>11</v>
       </c>
-      <c r="D14" s="58" t="inlineStr">
+      <c r="D14" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="F14" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F14" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="H14" s="68" t="inlineStr">
+      <c r="H14" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="J14" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L14" s="68" t="inlineStr">
         <is>
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="J14" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="M14" s="65" t="inlineStr">
+      <c r="N14" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="P14" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="R14" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="T14" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="V14" s="68" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="AV14" s="65" t="inlineStr">
         <is>
           <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="P14" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="R14" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="V14" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="AE14" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AH14" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="AJ14" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AS14" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AW14" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="AY14" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
         </is>
       </c>
     </row>
@@ -34034,24 +33920,34 @@
       <c r="B15" t="n">
         <v>12</v>
       </c>
-      <c r="D15" s="58" t="inlineStr">
+      <c r="D15" s="63" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="F15" s="58" t="inlineStr">
         <is>
           <t>MS A - 1</t>
         </is>
       </c>
-      <c r="F15" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="H15" s="68" t="inlineStr">
+      <c r="H15" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="J15" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L15" s="68" t="inlineStr">
         <is>
           <t>MS C - 1</t>
         </is>
       </c>
-      <c r="J15" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
+      <c r="N15" s="64" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
         </is>
       </c>
       <c r="P15" s="58" t="inlineStr">
@@ -34059,44 +33955,24 @@
           <t>MS A - 2</t>
         </is>
       </c>
-      <c r="R15" s="63" t="inlineStr">
+      <c r="R15" s="59" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="T15" s="63" t="inlineStr">
         <is>
           <t>MS B - 2</t>
         </is>
       </c>
-      <c r="V15" s="65" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="AE15" s="64" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="AH15" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="AJ15" s="63" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="AS15" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="AW15" s="68" t="inlineStr">
+      <c r="V15" s="68" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="AY15" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
+      <c r="AV15" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
         </is>
       </c>
     </row>
@@ -34549,119 +34425,129 @@
       <c r="B22" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="63" t="inlineStr">
+      <c r="C22" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 4</t>
+        </is>
+      </c>
+      <c r="E22" s="63" t="inlineStr">
         <is>
           <t>MS B - 6</t>
         </is>
       </c>
-      <c r="E22" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="F22" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="H22" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="I22" s="55" t="inlineStr">
+      <c r="F22" s="71" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="G22" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="H22" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="I22" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="L22" s="60" t="inlineStr">
+        <is>
+          <t>MD A - 5</t>
+        </is>
+      </c>
+      <c r="M22" s="55" t="inlineStr">
         <is>
           <t>MD V - 5</t>
         </is>
       </c>
-      <c r="J22" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="K22" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 3</t>
-        </is>
-      </c>
-      <c r="M22" s="66" t="inlineStr">
-        <is>
-          <t>WD B - 4</t>
-        </is>
-      </c>
-      <c r="N22" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="O22" s="62" t="inlineStr">
+      <c r="O22" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="Q22" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S22" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="U22" s="71" t="inlineStr">
+        <is>
+          <t>WD C - 3</t>
+        </is>
+      </c>
+      <c r="V22" s="58" t="inlineStr">
+        <is>
+          <t>MS A - 6</t>
+        </is>
+      </c>
+      <c r="Y22" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AA22" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="AB22" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 5</t>
+        </is>
+      </c>
+      <c r="AD22" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AF22" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AH22" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AI22" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 5</t>
+        </is>
+      </c>
+      <c r="AJ22" s="62" t="inlineStr">
         <is>
           <t>XD A - 4</t>
         </is>
       </c>
-      <c r="Q22" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="R22" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 4</t>
-        </is>
-      </c>
-      <c r="S22" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="T22" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 4</t>
-        </is>
-      </c>
-      <c r="W22" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="Z22" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="AA22" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 5</t>
-        </is>
-      </c>
-      <c r="AC22" s="67" t="inlineStr">
+      <c r="AL22" s="67" t="inlineStr">
         <is>
           <t>XD B - 4</t>
         </is>
       </c>
-      <c r="AE22" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 4</t>
-        </is>
-      </c>
-      <c r="AG22" s="65" t="inlineStr">
+      <c r="AP22" s="65" t="inlineStr">
         <is>
           <t>MD B - 5</t>
         </is>
       </c>
-      <c r="AI22" s="56" t="inlineStr">
-        <is>
-          <t>WD V - 4</t>
-        </is>
-      </c>
-      <c r="AJ22" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 6</t>
-        </is>
-      </c>
-      <c r="AM22" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 5</t>
+      <c r="AR22" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 5</t>
+        </is>
+      </c>
+      <c r="AT22" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 5</t>
         </is>
       </c>
     </row>
@@ -34669,104 +34555,104 @@
       <c r="B23" t="n">
         <v>2</v>
       </c>
-      <c r="D23" s="66" t="inlineStr">
-        <is>
-          <t>WD B - 3</t>
-        </is>
-      </c>
-      <c r="E23" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="F23" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="H23" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="I23" s="56" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="J23" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="K23" s="59" t="inlineStr">
-        <is>
-          <t>WS A - 3</t>
-        </is>
-      </c>
-      <c r="N23" s="57" t="inlineStr">
+      <c r="C23" s="55" t="inlineStr">
+        <is>
+          <t>MD V - 4</t>
+        </is>
+      </c>
+      <c r="E23" s="66" t="inlineStr">
+        <is>
+          <t>WD B - 4</t>
+        </is>
+      </c>
+      <c r="F23" s="71" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="G23" s="57" t="inlineStr">
         <is>
           <t>XD V - 2</t>
         </is>
       </c>
-      <c r="O23" s="62" t="inlineStr">
+      <c r="H23" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="I23" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="L23" s="71" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="M23" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="O23" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="Q23" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S23" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="V23" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 4</t>
+        </is>
+      </c>
+      <c r="Y23" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AA23" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="AD23" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AF23" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AH23" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AJ23" s="62" t="inlineStr">
         <is>
           <t>XD A - 4</t>
         </is>
       </c>
-      <c r="Q23" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="R23" s="53" t="inlineStr">
-        <is>
-          <t>MS V - 4</t>
-        </is>
-      </c>
-      <c r="S23" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="T23" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 5</t>
-        </is>
-      </c>
-      <c r="W23" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="Z23" s="58" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="AA23" s="56" t="inlineStr">
-        <is>
-          <t>WD V - 3</t>
-        </is>
-      </c>
-      <c r="AC23" s="67" t="inlineStr">
+      <c r="AL23" s="67" t="inlineStr">
         <is>
           <t>XD B - 4</t>
         </is>
       </c>
-      <c r="AE23" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 4</t>
-        </is>
-      </c>
-      <c r="AJ23" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 6</t>
-        </is>
-      </c>
-      <c r="AM23" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 5</t>
+      <c r="AR23" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 4</t>
         </is>
       </c>
     </row>
@@ -34774,69 +34660,84 @@
       <c r="B24" t="n">
         <v>3</v>
       </c>
-      <c r="D24" s="66" t="inlineStr">
-        <is>
-          <t>WD B - 3</t>
-        </is>
-      </c>
-      <c r="F24" s="62" t="inlineStr">
+      <c r="C24" s="61" t="inlineStr">
+        <is>
+          <t>WD A - 4</t>
+        </is>
+      </c>
+      <c r="F24" s="71" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="G24" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="H24" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="I24" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="L24" s="71" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="M24" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="O24" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="Q24" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S24" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="V24" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 4</t>
+        </is>
+      </c>
+      <c r="Y24" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AA24" s="62" t="inlineStr">
         <is>
           <t>XD A - 3</t>
         </is>
       </c>
-      <c r="H24" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="I24" s="56" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="J24" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="K24" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 4</t>
-        </is>
-      </c>
-      <c r="N24" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="Q24" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="R24" s="56" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="S24" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="W24" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AA24" s="56" t="inlineStr">
-        <is>
-          <t>WD V - 3</t>
-        </is>
-      </c>
-      <c r="AE24" s="62" t="inlineStr">
-        <is>
-          <t>XD A - 5</t>
+      <c r="AD24" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AF24" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AL24" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 3</t>
         </is>
       </c>
     </row>
@@ -34844,69 +34745,59 @@
       <c r="B25" t="n">
         <v>4</v>
       </c>
-      <c r="D25" s="71" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="F25" s="62" t="inlineStr">
+      <c r="G25" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="I25" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M25" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="O25" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="Q25" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S25" s="57" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="Y25" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AA25" s="62" t="inlineStr">
         <is>
           <t>XD A - 3</t>
         </is>
       </c>
-      <c r="H25" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="I25" s="56" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="J25" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="K25" s="60" t="inlineStr">
-        <is>
-          <t>MD A - 4</t>
-        </is>
-      </c>
-      <c r="N25" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="Q25" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="R25" s="56" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="S25" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="W25" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AA25" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
-        </is>
-      </c>
-      <c r="AE25" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 4</t>
+      <c r="AD25" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AF25" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AL25" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 3</t>
         </is>
       </c>
     </row>
@@ -34914,49 +34805,39 @@
       <c r="B26" t="n">
         <v>5</v>
       </c>
-      <c r="D26" s="71" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="F26" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 4</t>
-        </is>
-      </c>
-      <c r="J26" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="K26" s="71" t="inlineStr">
-        <is>
-          <t>WD C - 3</t>
-        </is>
-      </c>
-      <c r="N26" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="Q26" s="67" t="inlineStr">
+      <c r="G26" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="I26" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="M26" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="O26" s="67" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="R26" s="56" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="W26" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="AA26" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
+      <c r="Q26" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S26" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="AA26" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
         </is>
       </c>
     </row>
@@ -34964,34 +34845,34 @@
       <c r="B27" t="n">
         <v>6</v>
       </c>
-      <c r="F27" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 4</t>
-        </is>
-      </c>
-      <c r="J27" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="N27" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="Q27" s="67" t="inlineStr">
+      <c r="G27" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="I27" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="O27" s="67" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="R27" s="56" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="W27" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
+      <c r="Q27" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S27" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="AA27" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
         </is>
       </c>
     </row>
@@ -34999,24 +34880,29 @@
       <c r="B28" t="n">
         <v>7</v>
       </c>
-      <c r="J28" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="N28" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="Q28" s="67" t="inlineStr">
+      <c r="G28" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="I28" s="67" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="O28" s="67" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="W28" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
+      <c r="Q28" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S28" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
         </is>
       </c>
     </row>
@@ -35024,24 +34910,24 @@
       <c r="B29" t="n">
         <v>8</v>
       </c>
-      <c r="J29" s="68" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="N29" s="57" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="Q29" s="67" t="inlineStr">
+      <c r="G29" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="O29" s="67" t="inlineStr">
         <is>
           <t>XD B - 2</t>
         </is>
       </c>
-      <c r="W29" s="67" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
+      <c r="Q29" s="62" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S29" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
         </is>
       </c>
     </row>
@@ -35049,14 +34935,19 @@
       <c r="B30" t="n">
         <v>9</v>
       </c>
-      <c r="N30" s="70" t="inlineStr">
-        <is>
-          <t>MD C - 5</t>
-        </is>
-      </c>
-      <c r="W30" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 3</t>
+      <c r="G30" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="Q30" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="S30" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
         </is>
       </c>
     </row>
@@ -35064,9 +34955,19 @@
       <c r="B31" t="n">
         <v>10</v>
       </c>
-      <c r="W31" s="72" t="inlineStr">
-        <is>
-          <t>XD C - 3</t>
+      <c r="G31" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="Q31" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="S31" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
         </is>
       </c>
     </row>
@@ -35074,10 +34975,40 @@
       <c r="B32" t="n">
         <v>11</v>
       </c>
+      <c r="G32" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="Q32" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="S32" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" t="n">
         <v>12</v>
+      </c>
+      <c r="G33" s="70" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="Q33" s="72" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="S33" s="65" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -35344,6 +35275,186 @@
           <t>12:00</t>
         </is>
       </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="AG39" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="AH39" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="AI39" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="AJ39" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="AK39" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="AL39" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="AM39" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="AN39" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="AO39" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="AP39" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="AQ39" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="AR39" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="AS39" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="AT39" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="AU39" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="AV39" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="AW39" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="AX39" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="AY39" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="B40" t="n">
@@ -35458,6 +35569,376 @@
         <f>COUNTA(O40:P51)</f>
         <v/>
       </c>
+      <c r="P52">
+        <f>COUNTA(P40:Q51)</f>
+        <v/>
+      </c>
+      <c r="Q52">
+        <f>COUNTA(Q40:R51)</f>
+        <v/>
+      </c>
+      <c r="R52">
+        <f>COUNTA(R40:S51)</f>
+        <v/>
+      </c>
+      <c r="S52">
+        <f>COUNTA(S40:T51)</f>
+        <v/>
+      </c>
+      <c r="T52">
+        <f>COUNTA(T40:U51)</f>
+        <v/>
+      </c>
+      <c r="U52">
+        <f>COUNTA(U40:V51)</f>
+        <v/>
+      </c>
+      <c r="V52">
+        <f>COUNTA(V40:W51)</f>
+        <v/>
+      </c>
+      <c r="W52">
+        <f>COUNTA(W40:X51)</f>
+        <v/>
+      </c>
+      <c r="X52">
+        <f>COUNTA(X40:Y51)</f>
+        <v/>
+      </c>
+      <c r="Y52">
+        <f>COUNTA(Y40:Z51)</f>
+        <v/>
+      </c>
+      <c r="Z52">
+        <f>COUNTA(Z40:AA51)</f>
+        <v/>
+      </c>
+      <c r="AA52">
+        <f>COUNTA(AA40:AB51)</f>
+        <v/>
+      </c>
+      <c r="AB52">
+        <f>COUNTA(AB40:AC51)</f>
+        <v/>
+      </c>
+      <c r="AC52">
+        <f>COUNTA(AC40:AD51)</f>
+        <v/>
+      </c>
+      <c r="AD52">
+        <f>COUNTA(AD40:AE51)</f>
+        <v/>
+      </c>
+      <c r="AE52">
+        <f>COUNTA(AE40:AF51)</f>
+        <v/>
+      </c>
+      <c r="AF52">
+        <f>COUNTA(AF40:AG51)</f>
+        <v/>
+      </c>
+      <c r="AG52">
+        <f>COUNTA(AG40:AH51)</f>
+        <v/>
+      </c>
+      <c r="AH52">
+        <f>COUNTA(AH40:AI51)</f>
+        <v/>
+      </c>
+      <c r="AI52">
+        <f>COUNTA(AI40:AJ51)</f>
+        <v/>
+      </c>
+      <c r="AJ52">
+        <f>COUNTA(AJ40:AK51)</f>
+        <v/>
+      </c>
+      <c r="AK52">
+        <f>COUNTA(AK40:AL51)</f>
+        <v/>
+      </c>
+      <c r="AL52">
+        <f>COUNTA(AL40:AM51)</f>
+        <v/>
+      </c>
+      <c r="AM52">
+        <f>COUNTA(AM40:AN51)</f>
+        <v/>
+      </c>
+      <c r="AN52">
+        <f>COUNTA(AN40:AO51)</f>
+        <v/>
+      </c>
+      <c r="AO52">
+        <f>COUNTA(AO40:AP51)</f>
+        <v/>
+      </c>
+      <c r="AP52">
+        <f>COUNTA(AP40:AQ51)</f>
+        <v/>
+      </c>
+      <c r="AQ52">
+        <f>COUNTA(AQ40:AR51)</f>
+        <v/>
+      </c>
+      <c r="AR52">
+        <f>COUNTA(AR40:AS51)</f>
+        <v/>
+      </c>
+      <c r="AS52">
+        <f>COUNTA(AS40:AT51)</f>
+        <v/>
+      </c>
+      <c r="AT52">
+        <f>COUNTA(AT40:AU51)</f>
+        <v/>
+      </c>
+      <c r="AU52">
+        <f>COUNTA(AU40:AV51)</f>
+        <v/>
+      </c>
+      <c r="AV52">
+        <f>COUNTA(AV40:AW51)</f>
+        <v/>
+      </c>
+      <c r="AW52">
+        <f>COUNTA(AW40:AX51)</f>
+        <v/>
+      </c>
+      <c r="AX52">
+        <f>COUNTA(AX40:AY51)</f>
+        <v/>
+      </c>
+      <c r="AY52">
+        <f>COUNTA(AY40:AZ51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="C70">
+        <f>COUNTA(C58:D69)</f>
+        <v/>
+      </c>
+      <c r="D70">
+        <f>COUNTA(D58:E69)</f>
+        <v/>
+      </c>
+      <c r="E70">
+        <f>COUNTA(E58:F69)</f>
+        <v/>
+      </c>
+      <c r="F70">
+        <f>COUNTA(F58:G69)</f>
+        <v/>
+      </c>
+      <c r="G70">
+        <f>COUNTA(G58:H69)</f>
+        <v/>
+      </c>
+      <c r="H70">
+        <f>COUNTA(H58:I69)</f>
+        <v/>
+      </c>
+      <c r="I70">
+        <f>COUNTA(I58:J69)</f>
+        <v/>
+      </c>
+      <c r="J70">
+        <f>COUNTA(J58:K69)</f>
+        <v/>
+      </c>
+      <c r="K70">
+        <f>COUNTA(K58:L69)</f>
+        <v/>
+      </c>
+      <c r="L70">
+        <f>COUNTA(L58:M69)</f>
+        <v/>
+      </c>
+      <c r="M70">
+        <f>COUNTA(M58:N69)</f>
+        <v/>
+      </c>
+      <c r="N70">
+        <f>COUNTA(N58:O69)</f>
+        <v/>
+      </c>
+      <c r="O70">
+        <f>COUNTA(O58:P69)</f>
+        <v/>
+      </c>
+      <c r="P70">
+        <f>COUNTA(P58:Q69)</f>
+        <v/>
+      </c>
+      <c r="Q70">
+        <f>COUNTA(Q58:R69)</f>
+        <v/>
+      </c>
+      <c r="R70">
+        <f>COUNTA(R58:S69)</f>
+        <v/>
+      </c>
+      <c r="S70">
+        <f>COUNTA(S58:T69)</f>
+        <v/>
+      </c>
+      <c r="T70">
+        <f>COUNTA(T58:U69)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>